<commit_message>
release: finalize 1.3.0 documentation and explorer
Complete the MRIO explorer and database scope, review public download assets, add GLORIA annual readings, and recharacterise EXIOBASE GHG to the documented AR5 basis. Record the remaining add-sector compatibility fixes and release notes.
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/database_profiles/adb-62-economies-sets-06a54532.xlsx
+++ b/doc/source/_static/data/database_profiles/adb-62-economies-sets-06a54532.xlsx
@@ -1,12 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sets" sheetId="1" r:id="R9ee951fcfcc14693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="2" r:id="R3db4219465604e81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional memberships" sheetId="3" r:id="R35cb05d716b64615"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Sets" sheetId="1" r:id="R9ee951fcfcc14693"/>
+    <sheet name="Readings" sheetId="2" r:id="R3db4219465604e81"/>
+    <sheet name="Regional memberships" sheetId="3" r:id="R35cb05d716b64615"/>
+    <sheet name="Read me" sheetId="4" r:id="rId1"/>
+  </sheets>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14,105 +15,166 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
-    <x:numFmt numFmtId="200" formatCode="0"/>
-    <x:numFmt numFmtId="201" formatCode="@"/>
-    <x:numFmt numFmtId="202" formatCode="#,##0"/>
-  </x:numFmts>
-  <x:fonts count="5">
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="14"/>
-      <x:color rgb="FF202C38"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF566675"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF202C38"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Arial"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="3">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF245B6A"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="14">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="200" formatCode="0"/>
+    <numFmt numFmtId="201" formatCode="@"/>
+    <numFmt numFmtId="202" formatCode="#,##0"/>
+    <numFmt numFmtId="203" formatCode="@"/>
+  </numFmts>
+  <fonts count="9">
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF202C38"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF566675"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF202C38"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF302820"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF302820"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+  </fonts>
+  <fills count="6">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF245B6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF302820"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1"/>
+  </cellStyleXfs>
+  <cellXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="203" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0"/>
+  </cellStyles>
+</styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30791,4 +30853,108 @@
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae9258579ce74ef8"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/source_notice4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFF0783C"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="100" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
+      <c r="A1" s="20" t="str">
+        <v>Read me</v>
+      </c>
+      <c r="B1" s="20" t="str">
+        <v>ADB · 62 economies · economic accounts</v>
+      </c>
+    </row>
+    <row r="2" ht="15" hidden="0" customHeight="1">
+      <c r="A2" s="18" t="str">
+        <v>Contents</v>
+      </c>
+      <c r="B2" s="21" t="str">
+        <v>Native set labels and units. No economic observations, emission factors or coefficients.</v>
+      </c>
+    </row>
+    <row r="3" ht="15" hidden="0" customHeight="1">
+      <c r="A3" s="18" t="str">
+        <v>Verified years</v>
+      </c>
+      <c r="B3" s="21" t="str">
+        <v>2000, 2007, 2008, 2009, 2010, 2011, 2012, 2013, 2014, 2015, 2016, 2024</v>
+      </c>
+    </row>
+    <row r="4" ht="15" hidden="0" customHeight="1">
+      <c r="A4" s="18" t="str">
+        <v>How to use</v>
+      </c>
+      <c r="B4" s="21" t="str">
+        <v>Read Sets (or the named set tabs) for labels and units; Readings identifies source years. Identical inventories do not imply identical numerical results.</v>
+      </c>
+    </row>
+    <row r="5" ht="15" hidden="0" customHeight="1">
+      <c r="A5" s="18" t="str">
+        <v>Source</v>
+      </c>
+      <c r="B5" s="21" t="str">
+        <v>https://www.adb.org/what-we-do/data/regional-input-output-tables</v>
+      </c>
+    </row>
+    <row r="6" ht="15" hidden="0" customHeight="1">
+      <c r="A6" s="18" t="str">
+        <v>Attribution</v>
+      </c>
+      <c r="B6" s="21" t="str">
+        <v>Asian Development Bank</v>
+      </c>
+    </row>
+    <row r="7" ht="15" hidden="0" customHeight="1">
+      <c r="A7" s="18" t="str">
+        <v>Source terms</v>
+      </c>
+      <c r="B7" s="21" t="str">
+        <v>ADB Key Indicators data terms</v>
+      </c>
+    </row>
+    <row r="8" ht="15" hidden="0" customHeight="1">
+      <c r="A8" s="18" t="str">
+        <v>Terms URL</v>
+      </c>
+      <c r="B8" s="21" t="str">
+        <v>https://kidb.adb.org/terms</v>
+      </c>
+    </row>
+    <row r="9" ht="24" hidden="0" customHeight="1">
+      <c r="A9" s="18" t="str">
+        <v>Reuse</v>
+      </c>
+      <c r="B9" s="21" t="str">
+        <v>Credit ADB and the original dataset. Check the terms attached to the downloaded MRIO release; ADB Data Library has a separate CC BY 3.0 IGO policy.</v>
+      </c>
+    </row>
+    <row r="10" ht="15" hidden="0" customHeight="1">
+      <c r="A10" s="18" t="str">
+        <v>Changes</v>
+      </c>
+      <c r="B10" s="21" t="str">
+        <v>Extracted and arranged with MARIO. Native labels and units are retained. Country names and ISO matches are documentation metadata.</v>
+      </c>
+    </row>
+    <row r="11" ht="15" hidden="0" customHeight="1">
+      <c r="A11" s="18" t="str">
+        <v>Limit</v>
+      </c>
+      <c r="B11" s="21" t="str">
+        <v>A set inventory describes the parsed input, not the quality of the source or a licence to use its numerical data.</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>